<commit_message>
Update Jira performance report with complete paginated data
Fixed pagination by splitting queries into day-level and project-level
chunks to bypass the 100-result API cap. Complete data now captured:
- Previous Week Performance: 499 issues across 37 assignees (was 100)
- Current Week Assignments: 351 issues across 41 assignees (was 100)

https://claude.ai/code/session_017G1hi6ZhupGRoGRMmijRP8
</commit_message>
<xml_diff>
--- a/jira_performance_report_2026-05-14.xlsx
+++ b/jira_performance_report_2026-05-14.xlsx
@@ -470,13 +470,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,7 +515,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>AbdulRauf Siddiqui</t>
@@ -533,7 +533,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Ahmed Hussain Warwani</t>
@@ -547,11 +547,11 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Provide S3 links of updated videos to Uzair., Interview Of Ahmed Khan, Optimization of burgerlab server using multi-worker setup., crons to sync the insights are running every 15 minutes on burgerlab, Increase the time for all branches, URL open error on SPL Downtime Shell Select On-Prem server., setup TMS logger on all production wallet servers, Setup tms_stage index for elastic search stage</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>Setup tms_stage index for elastic search stage, setup TMS logger on all production wallet servers, Provide S3 links of updated videos to Uzair., Interview Of Ahmed Khan, Optimization of burgerlab server using multi-worker setup., crons to sync the insights are running every 15 minutes on burgerlab, Increase the time for all branches, URL open error on SPL Downtime Shell Select On-Prem server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Ali Hashim</t>
@@ -565,11 +565,11 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Multiple bill payments, issue with saved bills, update copies, Send QR and bank details with account receipts, Check if backend is getting analytics for onelink (Appsflyer), Change transaction message to utility - 3 variations, App copy - No internet / Transaction status pending, Change - Accounts banner copies and fix all CTA buttons, Remove Arshiya's access, KT, transfer of responsibilities, Remove Saddar's old page from restricted business portfolio, Edit video scripts for onboarding stories, Review business receipt copies, Task management and plan, Playstore creatives for UB, Video scripts for onboarding stories, Review assets for unbundl, T&amp;C copy for share and earn according to new design, New creatives on FB ads, Copies for UB for Categories, Invoices, PO, Filters, Share and earn banner CTAs, Share and Earn copy fixes, Update Urdu onboarding stories, Review Sale and Expense copy, Align Jira for the team, Fix onboarding stories, S&amp;E terms &amp; conditions look off, Test new build for product based PNs, App copies for udhaar, Push notifiaction changes and edits for share and earn, GA Funnel for Udhaar Blog, V1 of growth framework doc. Analyse and discuss with Fahad, New team mate's role and udhaar's plan with Fahad - Meeting, Push notifications for Share and earn and routing, Copy review and fixes, Saddar product push notifications, ads spend &amp; analyse FB ads weekly report</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>Edit video scripts for onboarding stories, Review business receipt copies, Task management and plan, Playstore creatives for UB, Video scripts for onboarding stories, Review assets for unbundl, T&amp;C copy for share and earn according to new design, New creatives on FB ads, Copies for UB for Categories, Invoices, PO, Filters, Share and earn banner CTAs, Share and Earn copy fixes, Update Urdu onboarding stories, Review Sale and Expense copy, Align Jira for the team, Fix onboarding stories, S&amp;E terms &amp; conditions look off, Test new build for product based PNs, App copies for udhaar, Push notifiaction changes and edits for share and earn, GA Funnel for Udhaar Blog, V1 of growth framework doc. Analyse and discuss with Fahad, New team mate's role and udhaar's plan with Fahad - Meeting, Push notifications for Share and earn and routing, Copy review and fixes, Saddar product push notifications, ads spend &amp; analyse FB ads weekly report, Multiple bill payments, issue with saved bills, update copies, Send QR and bank details with account receipts, Check if backend is getting analytics for onelink (Appsflyer), Change transaction message to utility - 3 variations, App copy - No internet / Transaction status pending, Change - Accounts banner copies and fix all CTA buttons, Remove Arshiya's access, KT, transfer of responsibilities, Remove Saddar's old page from restricted business portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Ali Iqbal</t>
@@ -583,11 +583,11 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Designed 4 mobile Play Store stories for Oscars (light mode)., Updated all copies across both mobile and tablet stories., Designed 4 mobile tablet Play Store stories for Oscars., Designed 4 mobile Play Store stories for Oscars (dark mode)., Spot &amp; Win Creative, Udhaar book reminder post with 2 supporting images, Targeting Rupin in this creative with 2 supporting images, Focusing on Udhaar book App (02 Udhaar book creatives for social media post 2 supporting images), Focusing on wallet (02 Udhaar book creatives for social media post 2 supporting images) , Design 01 Saddar billboard meme, with an engaging and relatable concept optimized for social media., Develop 02 Saddar catalog icon images, ensuring they are clean, scalable, and consistent with the design system., Create 02 Saddar web and in-app banners, optimized for both platforms with a cohesive look and feel., Design 02 Saddar catalog banner images, aligned with brand guidelines and visual consistency., Unbundle Creatives for Oscar, Saddar Product images thumbnail for videos, Social media creatives. (2 creatives + 4 supporting images), Saddar Product images thumbnail for videos, Design 5 Saddar Organic Social Post Creatives, Design Oscar Paid Ad Creatives — Restaurant Vertical (3-4 variants), Saddar social media creative with dimensions, Udhaar book carousel, Saddar Product images thumbnail for videos, Saddar App and web banner, Unbundle 8 Ads Creatives</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
+          <t xml:space="preserve">Design 01 Saddar billboard meme, with an engaging and relatable concept optimized for social media., Develop 02 Saddar catalog icon images, ensuring they are clean, scalable, and consistent with the design system., Create 02 Saddar web and in-app banners, optimized for both platforms with a cohesive look and feel., Design 02 Saddar catalog banner images, aligned with brand guidelines and visual consistency., Unbundle Creatives for Oscar, Saddar Product images thumbnail for videos, Social media creatives. (2 creatives + 4 supporting images), Saddar Product images thumbnail for videos, Design 5 Saddar Organic Social Post Creatives, Design Oscar Paid Ad Creatives — Restaurant Vertical (3-4 variants), Saddar social media creative with dimensions, Udhaar book carousel, Saddar Product images thumbnail for videos, Saddar App and web banner, Unbundle 8 Ads Creatives, Designed 4 mobile Play Store stories for Oscars (light mode)., Updated all copies across both mobile and tablet stories., Designed 4 mobile tablet Play Store stories for Oscars., Designed 4 mobile Play Store stories for Oscars (dark mode)., Spot &amp; Win Creative, Udhaar book reminder post with 2 supporting images, Targeting Rupin in this creative with 2 supporting images, Focusing on Udhaar book App (02 Udhaar book creatives for social media post 2 supporting images), Focusing on wallet (02 Udhaar book creatives for social media post 2 supporting images) </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Anwar Ahmed</t>
@@ -601,11 +601,11 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>add attachments list in invoice, discussion with QA and backend regarding business receipt, wallet receipt revamp deisgn and apis, complete functionality compatibilties of all the receipt, invoice and the success screen, Bank details card with QR code, Develop Business Receipt Screen revamp, Develop Invoice complete UI revamp and logic, Develop Business Success Screens (UI &amp; Logic)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>Bank details card with QR code, Develop Business Success Screens (UI &amp; Logic), add attachments list in invoice, discussion with QA and backend regarding business receipt, wallet receipt revamp deisgn and apis, Develop Business Receipt Screen revamp, Develop Invoice complete UI revamp and logic, complete functionality compatibilties of all the receipt, invoice and the success screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Asfand</t>
@@ -619,11 +619,11 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Smoke testing on beta, PO test cases verification, Quick sale copies verification, Quick sale desgin verification testing, Quick sale test cases verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
+          <t>Quick sale test cases verification, Smoke testing on beta, Quick sale copies verification, Quick sale desgin verification testing, PO test cases verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Ashhad Ahmed</t>
@@ -637,11 +637,11 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Banner Image, CTA Text and Description update, Loyalty &amp; Share-n-Earn Refund Refactor, Voucher Module R&amp;D &amp; API Integration, Django Form POS Reporting &amp; Dashboard UI Assets, Notification Resolvers &amp; Exclusion Logic, Batch Notification Engine &amp; Payload Integration, Create Django Form to Allow Agent to Download User POS Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
+          <t>Notification Resolvers &amp; Exclusion Logic, Batch Notification Engine &amp; Payload Integration, Loyalty &amp; Share-n-Earn Refund Refactor, Voucher Module R&amp;D &amp; API Integration, Django Form POS Reporting &amp; Dashboard UI Assets, Create Django Form to Allow Agent to Download User POS Data, Banner Image, CTA Text and Description update</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Asim Ur Rehman</t>
@@ -655,41 +655,545 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Get updated pull in my current branch and recheck all flow, Put Api in Add contact flow and category , Get Pull and update my current branch, Add contact  and category flow in wallet listing detail page</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
+          <t>Get Pull and update my current branch, Add contact  and category flow in wallet listing detail page, Put Api in Add contact flow and category , Get updated pull in my current branch and recheck all flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Ateeb Shaikh</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Issues Debug in Get Recharge Customer V1 , Wallet: Deactivate + Reuse after 99999 Logic,  Wallet: Virtual QR + Incoming Mapping, Wallet: Virtual IBAN Model and Generation API, Added Recent Transaction functionalty in backfuill recharge customer management command , Update Recent Transactions Cache After Successful Recharge,  Populate Recent Transactions In Customer Meta Model Through Management Command, Optimize Recharge APIs for customer level and transaction level, Add Missing Fields in Transaction APIs, Update the Recharge Api and Management Command to also include the Pagination supported Values in API and Managment Command, Save Recent Consumers and Pagination in Meta Model In Bill Payment API Successful Bill Payment,  Populate Recent Consumers and Pagination old meta thought management Command, Backfill and Update recent transactions of Test Users for Recharges and Bill Payments Management Command, Fixes and Test after PR Review, Fixes all recharges and bills new V3 APIs, Udhaar: Payment Settlement Integration, Udhaar: Khata Create/Delete Integration, Optimize Bills - Recent Consumers and Pagination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Aun Zaidi</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Anwar maqsood AI onboarding, Rupin app onboarding video (Shah Bhai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ayyan Bin Fawad</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Design Rupin brochure for distribution in market, Review product document for archival/recycle bin and share comments, Review document for accounts section redesign and share thoughts, Call 10 1bill users to gather feedback on why they prefer it to bank transfers, Listen to inbound calls and identify opportunities for application and improvement at agent level, Listen to customer conversion calls and identify issues faced in conversion, Call 10 users about feedback on how they manage stock levels(if they use stock in/stock out or manage inventory through invoices/POs), Call 10 users to ask what they use my accounts feature for and if they share accounts from there, Call 10 users on feedback about potential new features(recycle bin, dark mode, sms reminders, PNL), Call 10 users who saw stories but did not create Rupin account to see why they cancelled and if the feature would interest them, Share details on changes required/elements requested with Areeb, Design initial website for RUPIN using Oscar CMS elements, Transcribe customer conversion call recordings using eleven labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Bilal Ali Khan</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>RUPIN web copies, Udhaar Book (Playstore creatives), Oscar (Playstore creatives), Social Media Posts, Review copies given by Ammar Hashmi, Community Management, Udhaar Book Voiceover, March - social media performance report, Saddar Whatsapp Messages, Udhaar Book video voiceover, Content Calendar (Apr 2026), Research for outreach ideas for growth strategy, Growth strategy ideas, Facebook and Insta community management, Analysing Google Analytics dashboard for growth strategy, Rupin growth strategy, Oscar Creatives, Instagram creatives, Shoot employer branding video, Growth Discussion with team, Growth strategy doc., Commission video creative ideas, P&amp;L Slider - Edits, Push Notifcations, Unbundle Creative, Unbundl creatives for the themes (transparency, culture, utility), April Social media report, Shoot Udhaar Book video, Draft "Earn on Fuel" strategy for QR payments., Write an Employer Branding script, Saddar KT, Share and earn Marketing strategies</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Bilal Shaikh</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>CMS modifications for RUPIN, Accounting Review, Meeting for formulas, CMS modfification for Oscar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Hamza Naveed</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Cash Sales Difference in Z Report &amp; Sales Summary, Inventory Issue, Rockstar Vapor Issues, Converting All Dashboard Reports APIs from GET to POST with necessary changes required from query params to post data`, New Report: Basket Report, Moved all Dashboard Reporting to stage and fixes for some filters that occurred due to GET to POST, Filter out Settings in Settings API according to subtypes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Aamir</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>apply secrets manager on staging ec2 with limited permissions, create guide docs and update devops repo with script and implementation, analyze Servers Load avg and response time of APIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Sharjeel</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Shell Ev Station Complete Flow Creation, Zero Sales Report for Shell, Insight sale logs reporting on shell select, Foodpanda Margin Visibility for Shell</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Zain</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Design and implement Printer Setup page UI, Implement confirmation modal for image deletion, Create and design Edit Business Profile page UI, Design and implement Printers table UI, Implement “Printer Setup Successful” UI, Implement “Printer Test Successful” modal UI, Integrate available printer options into dropdown, Implement printer selection dropdown, Implement “Printer Drivers Installed Successfully” modal UI, Implement “Printer Software Installed Successfully” modal UI, Implement “Java Application Installed Successfully” modal UI, Remove Profile and Logout options from Business dropdown, Design and implement Backup Data page UI, Implement printer connect and disconnect functionality, Integrate available printers into table, Implement Create New PIN UI, Integrate current PIN verification functionality, Display error UI for incorrect PIN, Implement Enter Current PIN UI, Design and implement Change PIN page, Migrate existing backup functionality to new Backup page, Enable form submission on Enter key press across all Udhaar web forms, Integrate calculator-enabled input with full functionality in Quick Sale, Quick Expense, and Account Transactions forms, Tesing and bug fixing for PinCode section from Setting , Implement “PIN Updated Successfully” UI, Integrate new PIN update functionality</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Zeeshan</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>106</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Designing a YouTube Cover for Saddar Channel, Design Fast-casual Landing Page — Pain Points, Comparison, CTA Sections, Design Fast-casual Landing Page — Hero Banner &amp; Feature Icons, Design Fitness-centre Landing Page — Pain Points, Comparison, CTA Sections, Design Fitness-centre Landing Page — Hero Banner &amp; Feature Icons, Design Real-time-dashboard Landing Page — Pain Points, Comparison, CTA Sections, Design Real-time-dashboard Landing Page — Hero Banner &amp; Feature Icons, Design Multi location management Landing Page — Pain Points, Comparison, CTA Sections, Design Multi location management Landing Page — Hero Banner &amp; Feature Icons, Design Cafe Landing Page — Hero Banner &amp; Feature Icons, Design Cafe Landing Page — Pain Points, Comparison, CTA Sections, Design Vape Shop Landing Page — Pain Points, Comparison, CTA Sections, Design Vape Shop Landing Page — Hero Banner &amp; Feature Icons, Design Jewelry Landing Page — Pain Points, Comparison, CTA Sections, Oscar website images hotel section complete., Design Jewelry Landing Page — Hero Banner &amp; Feature Icons, Design Pharmacy Landing Page — Pain Points, Comparison, CTA Sections, Design Pharmacy Landing Page — Hero Banner &amp; Feature Icons, Design Clothing Landing Page — Pain Points, Comparison, CTA Sections, Design Clothing Landing Page — Hero Banner &amp; Feature Icons, Oscar website images Bakery &amp; Coffee section complete., 2 Instagram creative, 2 Instagram creative, Design Real Time Inventory Tracking Landing Page — Hero Banner &amp; Feature Icons, Design Real Time Inventory Tracking Landing Page — Pain Points, Comparison, CTA Sections, Design Loyalty Program Landing Page — Pain Points, Comparison, CTA Sections, Design Loyalty Program Landing Page — Hero Banner &amp; Feature Icons</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Nabeel Akram</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Set up read replicas for RNP and Udhaar RDS databases in a secondary region, so that database availability is maintained during failover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Rameez Javed</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Blogs, Revamp Old Blog, User Journey Udhaar Book &amp; Oscar, Blog, Revamp Old Blog, Optimize Saddar Category Page, App Store Listing Update, Overall Traffic Analysis, Write Oscar Blog: Best POS Software for Clothing Stores in Pakistan (2026), Write Oscar Blog: Best Pharmacy POS Software in Pakistan — FBR Integrated, Write Oscar Blog: FBR POS Compliance Guide for Pharmacies 2026, Revamp 2 Low-Performing Oscar Blogs (Rewrite + Internal Links + CTAs), Write Udhaar Blog: Best Business Wallet App in Pakistan for Small Businesses, Write Udhaar Blog: How to Open a Business Account Digitally in Pakistan, Write Udhaar Blog: Why Every Small Business Needs a Separate Business Account, Add CTAs &amp; Internal Links to Top 5 Udhaar Bill-Checking Blogs, Optimize Saddar Mobile Accessories Category Page, Update Oscar Play Store Listing — Description, Keywords, What's New, Update Udhaar Play Store Listing — Description, Keywords, What's New, AI Visibility Audit &amp; Strategy — Structured Data + AI Discoverability, Technical SEO Checks — GSC Indexing, Internal Links, Meta Fixes, SEO — Oscar Blogs, SEO — Udhaar Blogs, SEO — Udhaar CRO, SEO — Saddar On-Page, SEO — Play Store &amp; App Listings, SEO — AI Visibility, SEO — Technical, SEO Weekly Organic Sheet Update, Blogs, Old Blogs Update, Update WoW Organic Sheet, Udhaar Book User Journey, Blogs, Oscar Pharmacy Page Creation: KWs &amp; Copy, Oscar Blogs, Best Online Food Delivery Platforms in Pakistan (2026) — And How to Manage Orders with a POS, FBR POS Integration in Pakistan: Complete Guide for Businesses (2026), Best Restaurant Inventory Management Software in Pakistan (Reduce Wastage &amp; Increase Profit), Clothing Inventory Management: How Retail Stores Track Sizes, Stock &amp; Sales Efficiently, Oscar KW &amp; Tools Research, Oscar KW &amp; Tools Analysis, Weekly Organic Sheet Update, Organic sheet Update, Internal Linking, Link Oscar Blogs to Relevant pages, Blog: “What Is a Pharmacy? How Modern Pharmacies Manage Inventory, Billing &amp; Compliance”, KW Research and Weekly Planning , Link Oscar Blogs to Relevant pages, Blog: “Managing Inventory for a Boutique? Tools, Free Software &amp; When to Upgrade to a POS System”, Blog: "Boutique Inventory Management Made Simple: Best Tools, Free Software &amp; POS Solutions", Blog: “How to Start an Ecommerce Business in Pakistan (Without Inventory Chaos or Order Mistakes)”, Competitor Analysis Agent Creation &amp; Testing, Blog: “Why Most Ecommerce Businesses Fail in Pakistan (And How to Build One That Scales)”, Blog: “Pharmacy Billing Problems? How the Right Software Fixes Errors, Delays &amp; Compliance Issues”</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Saad Amin</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Smoke On Beta, Invoice Book Design Verification Testing, Invoice Book Test Cases Verification, Testing on Beta, Invoice Book Copies Verification, P&amp;L Test Cases Verification, P&amp;L Copies Verification, P&amp;L Design Verification Testing, Invoice Book Events Verification Testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Saad Saleem</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C12" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Backfill and Update recent transactions of Test Users for Recharges and Bill Payments Management Command, Fixes and Test after PR Review, Fixes all recharges and bills new V3 APIs, Update the Recharge Api and Management Command to also include the Pagination supported Values in API and Managment Command, Save Recent Consumers and Pagination in Meta Model In Bill Payment API Successful Bill Payment,  Populate Recent Consumers and Pagination old meta thought management Command, Udhaar: Payment Settlement Integration, Wallet: Deactivate + Reuse after 99999 Logic, Udhaar: Khata Create/Delete Integration,  Wallet: Virtual QR + Incoming Mapping</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="C25" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Quick smoke run on the stage build., Bug verification and quick smoke testing on beta., Creation of test cases for the Settings flow of UB Web., Design QA for the onboarding journey. , Copies verification for the business filter module., App design QA against the Figma design for the Business Filter module., Execute test cases for the Business Filter module., Design QA for the listing module., Execute test cases for the listing flow of business, Execute design QA and content verification for the expense module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Sadiya Tariq</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>16.09</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>CMS - Update Restaurant Page, April Strategy Evaluation for Restaurant Page, SEO Article - Ecommerce Review, Playstore Creatives Inspiration, Oscar Reservation Video Script, Clothing Page Organic Update, Restaurants page strategy (Version 2), Audit Website, SEO - Article Pharmacy Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Saim Khan</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Update Onboarding Funnel For New Release, Make Cohorts To Target &amp; Analyze, Make Funnel To See Drop Offs in Increase Limit Feature Within New Wallet, Develop Script To Split Customer MyAlice Conversation Into Actual Conversations, Add T1 and PU In The EMI Conversion File, Modify EMI Agent Performance Report To Add Breakdown Of Sheets Into New, Bookkeeping, And Wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Sami Amir</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Resolve Hubspot tickets, Fix sale report issue, Resolve hubspot tickets, Resolve HubSpot Tickets, Make changes as per review for new Bill updates, Review and test Bill new update PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Shah Zaman</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Udhaar Tutorials videos,  Publish on YouTube Channel, &amp; update Google Sheet, Udhaar Tutorials videos,  Publish on YouTube Channel, &amp; update Google Sheet, Saddar, China import Products Edit, Saddar, China import ZR Collection products shoot, Udhaar Tutorials (send money, bill payment and KYC), Udhaar Tutorials (Multiple bills pay), Saddar, China import products, Videos Uploaded on YouTube Channel, Saddar, China import Products Edit, Saddar, China import products shoot, Saddar, China import Products Edit, Edit Saddar videos, publish on YouTube, update Google Sheet, Audionic Products, Publish on YouTube, &amp; update Google Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shahzaib Ali</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Test the updated ORM queries on dataroom against the reported number, Research if we can update the existing ORM queries, Coordinate with Devops to setup logstash config for TMS logging, Create PR to merge TMS logging code to production, Finalize the architechture to implement, Analyze the composite index creation solution, Research for the best possible alternative solution, Finalize the architecture to update and optimize the script, Analyze existing backfill_recharge_customers command and plan optimization strategy, Enable TMS &amp; Monitor TMS alerts and validate log flow in Kibana/ELK, Test the effect of index creation, Implement optimized backfill_recharge_customers command, Finalize and document the complete step by step guide to create composite indexes, Review generated TMS alerts</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sohail Hussain</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>create task on jira, design review for onboarding, Tesing and bug fixing for Profile section from Setting , Implement Publish modal, Implement Image modal, Saddar return Order Detail UI, Implemented Verify Account screen, Implemented the New user signup B and its functionality, Implemented the New user signup A and its functionality, Implemented the Existing user signin and its functionality</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Syed Ammar Ali Hashmii</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Smoke testing on Beta, Discussion with zainab, saim &amp; shah bhai , 1st meeting with fahad bhai &amp; zainab, Review the document of Accounts unification, Quick Expense Design Verification Testing, Quick Expense Test Cases Verification, Write listing document, Wallet Onboarding Types &amp; Upgrade Limit – Discussion, Quick Expense Copies Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Syed Maroof Ali</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Set Ticket Creator in HubSpot When Creating Tickets via Django, PBX call recordingd</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Taha Hussain</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>PR Review: Update txn API, PR Review: Sync API, Bill Payment Earnings – Planning, PR Review: Bill Payment Earning Rule, Voucher Revamp - Planning, Voucher Revamp - DRC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Uzair</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Sale pos invoice number and invoice prefix fix for report, Raast unlink, Stock item visibility from sal pos, Fix - Customer report from account report collect reminder, Rest pin fix, Bill payment default customer view fix, AB Test for EMI stories video, image and page, Fix Space Input Issue in Bank Search Field on Send Money Screen, Customer Internal Layout Cleanup &amp; Scroll Behavior, Fix Space Input Issue in Bank Search Field on Send Money Screen, Accounts - Scrollable accounts customer supplier page, Wallet bill details screen consumer number fixed (Company name removed)., Wallet listing changes are done (contact name + consumer number) bill payment., Remove dekhein on wallet listing header., Remove shadow on Share &amp; Earn  banner., Share and earn: removed floating button on money., Sale and expense on-boarding video added., Screenshot and recording allowed., Recharge: removed summary from recharge listing and customer internal page., Recharge transaction cached., Recharge customer internal page pagination and architecture updated., Recharge search pagination and architecture updated., Recharge customer pagination, cached and architecture updated., Bill payment transaction label to"Transactions (all bills)"., Bill payment banner added on customer list., Bill payment floating button added., Bill payment transaction cached., Bill payment add customer fixed (Paying bill from customer internal and then add another bill from confirmation then customer was not showing)., Bill payment already paid bills fixed (Toast will show if bill already paid instead of add bill)., Bill payment consumers bill pagination and architecture updated., Bill payment consumers pagination and architecture updated., Bill payment search pagination and architecture updated., Bill payment customer pagination, cached and architecture updated., Offline remind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Wardah Fatima</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Pay Single Bill feature and other updates, Incorrect Filter Labels and Missing Amount Filter, “Organize Your Sales Transactions” Option Missing on P&amp;L Detail Screen, “Watch Video” Option Missing on P&amp;L Dashboard Board, Salary and Inventory Transactions Not Reflected in Profit &amp; Loss Report, View Transactions – “No Name” filter label incorrectly truncated showing only “N”, Tile Size Inconsistency When Switching Between Paid and Unpaid Status, Incorrect Slider Heading: "Add photo" should be "Attachment" in Expense PO., Tax and Discount Fields Allow Values Greater Than 100%, Field Label Inconsistency in Expense PO, View Transactions – Large amount and customer name overflowing transaction card, View Transactions – Day-wise transaction total missing beside day label, View Transactions – PDF icon missing from transactions screen, Add Expense – Device native keyboard appears along with app keypad causing overlap, Add Expense – Upload Attachment modal header mismatch with design, Add Expense – Incorrect “Sales” wording in status nudge content, Add Expense – Missing QR code on receipt and incorrect tab label, Add Expense – Bill number not incrementing for multiple expenses, Order Discount Validation Issue &amp; UI Overlap on Input Field, Payment Method Field Appears Empty on Invoice Screen, Title: No Options Available When Selecting “All Payment Methods” and “Status” Filters, Add Expense – Category – “See More” displayed as button instead of link text, Incorrect Total Calculation with Tax and Discount on Invoice, Add Expense – Amount field focus and cursor position resets incorrectly., Missing "Subtotal" text in Quick Sale summary; only numeric value is visible., User Navigates Back Instead of Staying on Confirmation Modal in Invoice Flow, Filters – Category accordions do not support multiple open states simultaneously, Filters – Status – Multi-selection not working for Paid and Unpaid options, Filters – Payment Method – Multi-select not working despite checkbox UI, Filters – Category – Selected category not shown in header summary text, Quick Sale: Custom app keypad remains visible while scrolling., Edit Invoice Option Missing, Expense - PO - Missing Line Item Total Calculation, Incorrect Discount Calculation in Rupees (Applies 1% Instead of Entered Value), Staff Book Back Icon Missing on Quick Actions Screen, Incorrect Validation and Digit Limit Issue in Invoice Amount Field, View Transactions – Inconsistent expense abbreviation (Bill vs EXP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Zainab Hanif</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Wallet home screen design V2 , add money redesigned v1, Research, reviewing user feedback and formatting document for wallet home (redesign), Design components for wallet &amp; business receipt, trx details and confirmation , Finalizing design flows for new wallet design, Screen design for no internet in between wallet transaction, Upgrade account - design v1, Upgrade account- research , Design for customize rupin card, research on customize rupin card, Design for account limit, Research on account limit , Upgrade account design v2, add money redesigned v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Zubair</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Stock book Feedback V-2 , Multi bills payment fixes - V2, Stock book Feedback - V1, Multi bills payment fixes, Wallet - Internal listing changes, Voucher - Filters (Main + Slider), Bill payment - Filters (Main + Slider), Easyload - Filters (Main + Slider), Wallet  - Filters (Main + Slider), Listing for Business transactions, Listing for Wallet transaction, Stock changes, Stock Filter - Main + Slider</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>maroob</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Add Payment method selection options for Restuarants order screen, prepayment bill calculations discount and subtotal fixes and deploy to prod , Test cases Execution 251 to 473, Test cases Execution 1 to 250, R&amp;D for receipt customization and payment method tax selection, Reciept and prepayment slip fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>muhammad Ubaid</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Order Data Handling &amp; Edge Cases  Items mapping, Order Details API Integration Fetch single order, Handle Order Filters / Search, Order History API Integration, Map &amp; Handle Credit History Data , Credit History API Integration Fetch payment history, Handle Pay Credit Flow Logic , Implement Pay Credit API Integration  Submit credit payment, Error &amp; Edge Handling for Details Screen  Missing fields Partial data, Handle Credit Data Logic  Credit balance Validation, Handle Loyalty Points Logic Available points Mapping &amp; formatting, Customer Details API Integration Fetch single customer data, Handle Non-Ideal States, Debounce Search Optimization  Prevent excessive API calls, Implement Filters (if API supports)  Example: visits / date, Implement Search API Integration   Search by name/phone, Handle Empty / No Data State  No customers API failure fallback, State Management for Customer List  Loading Success Error, Handle Pagination  Page, limit handling Load more / next page, Implement Customer List API Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>283.75</v>
-      </c>
-      <c r="D13" s="6" t="inlineStr"/>
+      <c r="B41" s="6" t="n">
+        <v>499</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>1200.24</v>
+      </c>
+      <c r="D41" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -706,13 +1210,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -751,43 +1255,43 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>AbdulRauf Siddiqui</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">add CSV method for manual call logs, Add call classification in recordings., Accounts, In/Out, Sale POS, Invoice Report Fixes, PBX Manager Dashboard, AI Whatsapp chat support </t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
+          <t>AI Whatsapp chat support , Accounts, In/Out, Sale POS, Invoice Report Fixes, PBX Manager Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Ahmed Hussain Warwani</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Interview of Muhammad Rehan Khan, Establish site-to-site VPN connectivity for partners in the secondary region, so that external integrations remain accessible during outages., research and setup roll back functionality on bitbucket pipelines., Coordination with Wateen to get the CIR connection for RAAST</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>research and setup roll back functionality on bitbucket pipelines., Establish site-to-site VPN connectivity for partners in the secondary region, so that external integrations remain accessible during outages., Interview of Muhammad Rehan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Ali Hashim</t>
@@ -801,11 +1305,11 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>PNs to new wallet completed (no txn) and abandoned process, Convert users searching Check Bill - Strategy and design changes, Onboarding video review, Udhara book / Rupin new listing (images), Oscar playstore images, Oscar videos coordination, Share requirements for building an in-house push notification tool, Call new wallet abandoned / successful customers for feedback, Sort onesignal pricing and plan, Share plan for V1 of growth plan, Call new wallet abandoned / successful customers for feedback, Playstore creatives for UB</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>Call new wallet abandoned / successful customers for feedback, Sort onesignal pricing and plan, Share plan for V1 of growth plan, Call new wallet abandoned / successful customers for feedback, Share requirements for building an in-house push notification tool, Onboarding video review, Udhara book / Rupin new listing (images), Oscar playstore images, Oscar videos coordination, PNs to new wallet completed (no txn) and abandoned process, Convert users searching Check Bill - Strategy and design changes, Playstore creatives for UB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Ali Iqbal</t>
@@ -823,25 +1327,25 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Anwar Ahmed</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>wallet listing revamp new filters flow revamp, wallet listing revamp add contact flow, wallet listing revamp functionality , wallet listing ui revamp complete, wallet listing revamp discussion with backend, events integration for wallet and business receipt, test cases for wallet and business receipt entire flow, new icons installation for wallet and business receipt entire flow, Business and wallet receipt and success screen revamp and wallet listing revamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>Business and wallet receipt and success screen revamp and wallet listing revamp, events integration for wallet and business receipt, test cases for wallet and business receipt entire flow, new icons installation for wallet and business receipt entire flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Areeb Sheikh</t>
@@ -859,25 +1363,25 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Arshiya</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>30</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Call customers for video review, Facebook community managment, Facebook community managment, qoura posting, facebook community managment, earbuds and smartwatch catalogue creative, saddar post ideation, Facebook community managment, Saddar social media creative post &amp; website banner, Qoura posting, Collect Text/Video Testimonials from Repeat Customers, Send WhatsApp Marketing Blast with Impromptu Videos, Create Saddar Organic Social Content Plan &amp; Post 5 Times, Identify &amp; Reach Out to 2-3 Influencers, Plan Saddar marketing Strategy, Plan &amp; Shoot 2-3 Impromptu WhatsApp Marketing Videos, Audit &amp; Remove Poor-Reviewed Products, Set Up Abandoned Cart WhatsApp Auto-Messages, Banners ideation for Saddar, saddar social media 5 post, Plan Saddar marketing Strategy</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
+          <t>Call customers for video review, Facebook community managment, Facebook community managment, qoura posting, facebook community managment, earbuds and smartwatch catalogue creative, saddar post ideation, Facebook community managment, Saddar social media creative post &amp; website banner, Qoura posting, Collect Text/Video Testimonials from Repeat Customers, Send WhatsApp Marketing Blast with Impromptu Videos, Create Saddar Organic Social Content Plan &amp; Post 5 Times, Identify &amp; Reach Out to 2-3 Influencers, Plan Saddar marketing Strategy, Plan &amp; Shoot 2-3 Impromptu WhatsApp Marketing Videos, Audit &amp; Remove Poor-Reviewed Products, Set Up Abandoned Cart WhatsApp Auto-Messages, Banners ideation for Saddar, saddar social media 5 post</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Asfand</t>
@@ -895,7 +1399,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Ashhad Ahmed</t>
@@ -909,59 +1413,599 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Integrate Redeem Points into Voucher Purchase Flow, Implement Points Deduction &amp; Calculation Logic, Implement Points Validation Logic for Redemption, Add redeem_points Flag to Buy Voucher API, Implement Business Logic for purpose Handling, Add purpose Field to Buy Voucher API, Voucher API'S Development Doc, Identify File-Based Fields in Udhaar &amp; Wallet Microservice and Migrate Storage to S3 for DR Readiness, Integrate Coins Flow into Voucher Purchase API, Implement Coins Business Logic in Voucher System, Add Coins Fields &amp; Database Schema Updates, Implement Popular Voucher API v2 Endpoint, Define Popular Voucher API v2 Contract &amp; Schema, Voucher Revamp – API Enhancements and Feature Updates</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
+          <t>Integrate Coins Flow into Voucher Purchase API, Implement Coins Business Logic in Voucher System, Add Coins Fields &amp; Database Schema Updates, Implement Popular Voucher API v2 Endpoint, Define Popular Voucher API v2 Contract &amp; Schema, Voucher Revamp – API Enhancements and Feature Updates, Identify File-Based Fields in Udhaar &amp; Wallet Microservice and Migrate Storage to S3 for DR Readiness, Integrate Redeem Points into Voucher Purchase Flow, Implement Points Deduction &amp; Calculation Logic, Implement Points Validation Logic for Redemption, Add redeem_points Flag to Buy Voucher API, Implement Business Logic for purpose Handling, Add purpose Field to Buy Voucher API, Voucher API'S Development Doc</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Asim Ur Rehman</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Update All categories logic with selected language in wallet flows, wallet permissions flow for accepted user , Remove Api from easyload customer for get total recharge and total commision, Update Detail pages of wallet listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ateeb Shaikh</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Send money refund can only be given either if the transaction is not in sessions report or its not in both unreconciled and kibana rnp logs., Integration with Bill Payment Flow + Validation Layer, Consumer Number Extraction Engine (Biller-aware parser), QR Payload Extraction API Integration, Biller QR Format Discovery &amp; Mapping Design, Testing, Refund + Reconciliation Workflow, Settlement Report Validation Logic, Admin Panel + Manual Control, Create the new Model to store the Rejected Transactions, Create dedicated URL flow for .get()-based partner API views and regression-test behavior., Identify views using .get() on async tasks that trigger partner API calls., Validate and fix late-fee refund behavior for failed bill payments., Audit and refactor async tasks that use Django Client/APIClient to call internal views., Address the Errors if any Bank Faces while Scanning the QR, Test the QR with Every Bank, Create the new QR with only the Required Tags , Identify the Extra Tags in our QR according to the SBP QR Documentation, Limits for test users to be capped at 5k per month and 1000 per transaction., If a payable object is scheduled but not running, then a new payable can be created from the payables ledger action. Once new payable is created, previous payable will be marked as complete., Bills should be allowed to be paid even after due date, as long as 1link confirms that the bill can be paid., Fix amount comma issue in notification, Rupin Account should come up on top when returning account search results, Review and reduce the QR code size and test the new QR by paying via main stream banks</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Aun Zaidi</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Create Short-Form Cuts of All 4 Videos for Social Media, Edit Pharmacy Client Testimonial — Final Cut, Edit Clothing Client Testimonial — Final Cut, Generate Clothing Demo Video with Ai— Final Cut, Edit Clothing Store Demo Video — Final Cut, Shoot Client Testimonials — Clothing + Pharmacy Owners (On-Site), Rupin onboarding video (female version), Onboarding videos, Onboarding videos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Ayyan Bin Fawad</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Customer Conversion Management, Customer calls, Rupin Stockbook Redesign, Analyze customer feedback and create Stockbook Redesign Document, Review upcoming features, Create plan using Claude and transcribed calls to increase growth from Saddar calls, Transcribe calls from Saddar agents using Notebook LLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Bilal Ali Khan</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Calls to consumers, Oscar Playstore screenshots., Copies, Call to consumers, Check Bill plan, Social media posting, Community management, Instagram activity follow up, Consumer calls, V1 Growth document, Share and Earn GTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Bilal Shaikh</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="4" t="n">
-        <v>64.5</v>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>wallet permissions flow for accepted user , Update All categories logic with selected language in wallet flows, Remove Api from easyload customer for get total recharge and total commision,  Update Detail pages of wallet listing, Update All detail pages of Business Tools (Quick sale and expense, invoice, purchase order , sale pos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Ateeb Shaikh</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bills should be allowed to be paid even after due date, as long as 1link confirms that the bill can be paid., Limits for test users to be capped at 5k per month and 1000 per transaction., If a payable object is scheduled but not running, then a new payable can be created from the payables ledger action. Once new payable is created, previous payable will be marked as complete., Integration with Bill Payment Flow + Validation Layer, Consumer Number Extraction Engine (Biller-aware parser), QR Payload Extraction API Integration, Biller QR Format Discovery &amp; Mapping Design, Testing, Refund + Reconciliation Workflow, Settlement Report Validation Logic, Admin Panel + Manual Control, Create the new Model to store the Rejected Transactions, Create dedicated URL flow for .get()-based partner API views and regression-test behavior., Identify views using .get() on async tasks that trigger partner API calls., Validate and fix late-fee refund behavior for failed bill payments., Audit and refactor async tasks that use Django Client/APIClient to call internal views., Address the Errors if any Bank Faces while Scanning the QR, Test the QR with Every Bank, Create the new QR with only the Required Tags </t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="C18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Discussed Accounting APIs, Vendor Bills PO to Bill, Dashboard P &amp; L, Aramco report testing, Oscar AI adjustments</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Hamza Naveed</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect validation message shown on partial payment in Pay Credit flow, Incorrect validation message displayed when entering 0 amount in Pay Credit modal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Aamir</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Develop a script that validates DR site health (databases, VPN connectivity, and service availability) during drills, so that we can confirm all systems are functioning correctly after failover., Configure Redis dump for Udhaar core cache and wallet cache, so that cache data can be restored in case of failure., Setup ubuntu server on PC for oscar, Custom CI/CD pipeline for just code update on all prod servers., Apply security headers to cobu all 3 domains, Create pipeline for website cms prod, setup cobu-api on Singapore region</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Sharjeel</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Happy Hour Reporting on central Shell</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Sheheryar Izhar</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Wallet listing updates, Bill payment flow - udhaar blog, Care Form Requirements, Setup an upload routine for refunds data processed by Recon team. This refunds data would then automatically process the pending refunds., SMS Bundle Development PR Changes and Test, Fixed Existing Oscar API's</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Muhammad Zain</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Implement business overview cash flow test cases, Implement uncategorized page main non ideal, Implement export invoice test cases, Implement send reminder test cases, Implement delete invoice test cases, Implement edit invoice test cases, Implement record payment test cases, Implement sale invoice add discount and tax test cases, Implement sale invoice create invoice test cases, Implement sale invoice non-ideal test cases, Remove sidebar from new business form authorized user flow, Implement Sale POS (Udhaar payment flow) test cases, Implement Sale POS (Stock list cash flow)	 test cases, Implement Sale POS (Draft sales) test cases, Implement Sale POS (Edit open item name) test cases, Implement Sale POS (Add customer, Add discount, Add tax, Open item cash flow) test cases, Implement Sale POS non ideal test cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Nabeel Akram</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Create an DR drill playbook that includes all DevOps steps and validation scripts, so that disaster recovery procedures can be executed consistently and efficiently., Implement a monthly backup policy for critical EC2 instances in the secondary region, so that systems can be recovered when needed., Provision a DR S3 bucket for Udhaar web assets and configure cross-region replication with the primary bucket, so that web content remains available during regional failures., Define and configure security groups for all compute and database resources in the secondary region, so that network access is properly controlled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Rameez Javed</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Oscar Blogs  , Oscar Copies KWs, Competitor Analysis Agent Creation and testing, Internal Linking, Organic sheet Update, Oscar Blogs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Saad Amin</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Test on stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Saad Saleem</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>View Transactions – Minor UI jerk observed when navigating from “See More” to transaction listing, Content verification for the purchase order module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Sadiya Tariq</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Rupin Research Study, Demo Restaurant Video Feedback, Instagram Archive Posts, Instagram Profile Update, Linkedin Follower Revival Internal, Instagram Followers Revival Internal, Creatives/Review Website</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Saim Khan</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Wallet Adoption Project: Convert Bookkeeping Users To Wallet, AI Agent For EMI Analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Sami Amir</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Capture selfie image on account opening, no need to show on the account opening page., Optimize billings APIs, Enable deletion of test users from user docs. Only test users can be deleted on production. Test users may be retrieved from the environment file., Optimize Billing customer and transaction APIs, Optimize Recharge customer and transaction APIs, Optimize listing APIs for customer level and transaction level, test task hubsport flow, When transliteration API fails, Idenfo profiles should not be created, DB-Driven Mock API Framework for Staging (Postman Import Support)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Samin Jilani</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Daypart filters dashboard - API based dynamic filters on listings on dashboard, Daypart filters - create day part filter flow, Daypart filters - settings panel and screen work, Setting toggle work on list , Pre/Post Discount Tax Calculation Fix, App consistency work- Tax and split bill app changes, Split Bill (Payment Method Tax fixes), Make a searchable dropdown for reports header, Discount calculation fix on Post discounted tax setting, Post discount tax fixes, Prioritize order level tax over payment method tax, Line level discount and tax tweaks, pos core consistency work, Service type products work , Quantifable modifiers work, Tax by payment method in app, Split bill consistency work in app, Discounts consistency work, Taxes consistency work in app, Discount fix on post discounted tax, Subtotal fix on post discounted tax, ., Enable payment methods selection for each splitted payment., Observe edge cases of split bill, Discussion with team, research on how split bill should work and how will taxes and discounts behave., Observe architecture changes and formulate a solution, Lock taxes on split payments, Side navigation bar opens when user clicks on Recall Order, Dine-in orders not displayed after applying Dine-in filter in KDS History, Break order level discount to line level for cleaner calculations</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Shah Zaman</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Products Videos Uploaded on YouTube Channel &amp; videos links update, China Import ZR Collection Product Photoshoot, Saddar YouTube Channel Cover Design, ZR Collection Products Editing, Saddar, China Import  ZR Collection Product Shoot , Saddar, China import products, Videos Uploaded on YouTube Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Shahzaib Ali</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Activate TMS on Production and monitor the alerts, R&amp;D for risk scoring and enhancing tms using the risk score, Test the updated APIs, Create permission class and add in the required APIs, Add required models, Update and optimize backfill script to make sure that customer transaction table contains bills/vouchers and does it fast., Merchant Account Action to be immutable except for status and comments or required fields., Update multi user sync APIs according to recent changes and coordinate with frontend, Introduce a risk model based on Idenfo data and internal metrics provided by the Compliance team, Introduce other factors into transaction monitoring system</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Sohail Hussain</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Rupin - Onboarding, New Onboarding First screen with animation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Syed Ammar Ali Hashmii</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Design QA for Stock Book</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Syed Maroof Ali</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Multiple Sprint Issue in HR System, Implement settings printer section test cases, HubSpot X Jira Integrations, Claude Agents For EMI Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Taha Hussain</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>PR Review: AWS secret manager, PR Review: SMS Bundle Updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Uzair</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>View Transactions – Missing loader indicator on scroll for pagination, Filters – Category – Categories not translated in Urdu language, Global UI: QR code central logo appears in square block instead of round., Disable page-level scrolling for QR Receipt screen and fix banner position, Wallet details page on send money: Account title fixed, Send money polling failed due to internet fixed., Voucher polling failed due to internet fixed., Recharge customer routing fixed., Recharge polling failed due to internet fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Waleed</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Fix and consistent loaders in all udhaar web, Fix font size inconsistencies in title text boxes across the application, update the filter view of transation list, Update the structure and UI of the Bill Payment, Easyload, Packages, and Vouchers detail screens., Update the structure and UI of the Transaction screen., Update the structure and form components of the Vouchers screen., Update the structure and form components of the Easyload screen., Update the structure and form components of the Bill Payment screen., Update the structure and UI components of the Send Money screen., Update the structure and UI components of the Load Money screen., Create a unified list for Earn Money, Bill Payments, and Vouchers, and update the table structure and UI according to the new design, Update the All Transactions screen filter view UI and structure according to the new design</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Wardah Fatima</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Quick Expense - Send Money – Beneficiary selection shows loader only and leads to dead end (flow blocked), List Screen – Missing pagination loader causing stuck and non-smooth scrolling experience, Quick Sale: 'Add contact' button does not update to show selected contact., Incorrect Currency Name Displayed in Toast Message on Currency Selection, Quick Sale: Native keyboard overlaps custom app keypad on numerical fields., Quick Expense – Notes field triggers calculator and native keyboard causing input loop behavior, Quick Sale: Order discount toggle button and tapping area are too small., Quick Expense – Cursor jumps to “Rs.” prefix on tapping amount field after entry, Quick Expense – Red underline appears below “Rs.” when entering amount, Camera Not Opening When Scanning Barcode on Invoice Screen, Quick Sale: Tax and discount percentage field allows values greater than 100%., Quick Sale: 'Notes' field is hidden behind the keyboard., Quick Sale: Amount field only displays 8 digits (should be 12)., Quick Sale: System allows negative amount entries., Restrict Edit &amp; Delete for QR Received Payments and Send Money Transactions, Make Header Tab Scrollable with Content, Amount Overflow in Listing View – Not Truncating, Adjust P&amp;L Amount Font Size for Large Values, Add Expense – Save button missing border as per design, Filters – Week date filter returning transactions outside selected range, Filters – Incorrect results when combining Payment Method, Status, and Contact filters, Upload Image Modal UI Mismatch (Header Text, Option Order, and Labels Incorrect), "Quick Sale" module fails to enforce the 10-file attachment limit., Filters – Date (Urdu) – Inconsistent translation for “Past” text, Layout "jumps" or changes size when toggling between Paid and Unpaid in Quick Sale., Incorrect Navigation After Saving New Item Added via Barcode Scan in Invoice Book, Filters – Unapplied filters get applied on back navigation without tapping Apply, Filters – Amount – No input length validation allowing excessive number entry, Subtotal Text Missing on Invoice Book While Adding Items, Transaction Listing – View filter spacing issues in modal layout, Filters – View &amp; Amount – Checkmark icon size mismatch and extra spacing in currency format, Filters – Icons are inconsistent in size, Quick sale - View transactions - Filter Label Truncation: "No name" contact filter displays as "N" in active filter tile., Transactions: All transactions in listing display identical ID 'INV#1'., Quick sale - Invoice: Payment method appears empty when 'Bank Paid' is selected., Quick Sale: 'Update amount' toggle is partially hidden behind the 'Next' button., Quick Sale: 'See more' button in Category section is missing proper styling., Test cases, Events, Copies, Test cases, Events, Copies, Integrate updated save bill functionality., Add contact flow., View save bill listing and it’s detail modal., No Results Found” Screen Briefly Appears Before Transaction List on “See More” Click, Non-ideal screens must not include a back button in the header., "Undefined" displayed in Name and Account Number fields below QR code for guest users., Filters – Incorrect results when combining multiple filters with Amount range, Quick sale - Language Urdu/Roman - The content appearing below Unpaid toggle need to change as per selected language, Insufficient spacing between Urdu text labels and radio buttons in Quick Sale module., Add Expense – “Add Contact” text not updating after contact selection, Add Expense – Category label not updating after selection, Clickable Area Extends Outside “See Details” Text, Screen Jerks When Dismissing “Transaction Add Kar Ke P&amp;L Dekhen” Modal by Tapping Outside, Unable to Add Contact from Transaction Option on P&amp;L Main Page, Deleted Transaction Does Not Remove Immediately Until Navigating Back, Update Missing Content as per Attached File, Incorrect Decimal Formatting in “Payment Received” Field (Multiple Zeros After Decimal), Signature Not Displayed in Preview and Final Invoice, Filters – Filter option visually shrinks on tap interaction, View Transactions – Scroll lag and blank screen observed during fast scrolling, View Transactions – Missing space after abbreviations (Bill, PO, INV, POS), View Transactions – Filter icon background shape mismatch and missing search icon, Missing Content Not Updated as per Attached File, "Watch Video” Option Not Clickable on P&amp;L Detail Page Graph Section, Discount Value Showing as 0 on Receipt, Uploaded PDF Appears Blank in Invoice Attachments</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Zainab Hanif</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Formatting document for design as per user req with ayan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Zubair</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Return Flow - Research document , Review Accounts document, Recycle bin / archival, Stock book feedback - V1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>maroob</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Accounting APIs Integration &amp; FE, oscar.pk Fixes, Error handling and Filter implementation , update pdf export template according to API data , balance sheet API integration , P &amp; L Api integration, Categories &amp; Items Text is Not Displayed in Sentence Case in POS Default View</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>muhammad Ubaid</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Customer creation date is not displayed in Summary &amp; Detail section for newly created customers, Customer name and order count are not displayed on Customer Summary &amp; Detail screen header, Loyalty points are calculated incorrectly for customers across orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>366.5</v>
-      </c>
-      <c r="D15" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="n">
+        <v>351</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>788.75</v>
+      </c>
+      <c r="D45" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>